<commit_message>
Bump to 1.0.0.9001 and renew PubGeneticResource livestock batches.
Document the shared type vocabulary for crop/microbe and livestock notices, and ship the 2021-2023 YAML pipeline with the updated dataset.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/data-raw/data-tidy/public-site/moa-genetic-resource/xlsx/list-year-2024-batch-03.xlsx
+++ b/data-raw/data-tidy/public-site/moa-genetic-resource/xlsx/list-year-2024-batch-03.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\github\techme\data-raw\public-site\moa-genetic-resource\xlsx\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\github\techme\data-raw\data-tidy\public-site\moa-genetic-resource\xlsx\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6E4E1EC4-7CD4-43F0-8602-7E8C43AA5684}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A936C478-AD9D-42C0-A8C4-23DC4726E3CF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="51480" yWindow="5070" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet 1" sheetId="1" r:id="rId1"/>
@@ -174,10 +174,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>畜禽</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <r>
       <rPr>
         <sz val="11"/>
@@ -441,6 +437,10 @@
   </si>
   <si>
     <t>贵州</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>畜禽保种场</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -1015,19 +1015,19 @@
         <v>32</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>33</v>
+        <v>66</v>
       </c>
       <c r="D9">
         <v>1</v>
       </c>
       <c r="E9" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="F9" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="F9" s="1" t="s">
-        <v>35</v>
-      </c>
       <c r="G9" s="2" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
     </row>
     <row r="10" spans="1:7" ht="16.5" x14ac:dyDescent="0.3">
@@ -1038,19 +1038,19 @@
         <v>32</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>33</v>
+        <v>66</v>
       </c>
       <c r="D10">
         <v>2</v>
       </c>
       <c r="E10" t="s">
+        <v>35</v>
+      </c>
+      <c r="F10" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="F10" s="1" t="s">
-        <v>37</v>
-      </c>
       <c r="G10" s="2" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
     </row>
     <row r="11" spans="1:7" ht="16.5" x14ac:dyDescent="0.3">
@@ -1061,19 +1061,19 @@
         <v>31</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>33</v>
+        <v>66</v>
       </c>
       <c r="D11">
         <v>3</v>
       </c>
       <c r="E11" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="F11" t="s">
         <v>38</v>
       </c>
-      <c r="F11" t="s">
-        <v>39</v>
-      </c>
       <c r="G11" s="2" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
@@ -1084,19 +1084,19 @@
         <v>31</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>33</v>
+        <v>66</v>
       </c>
       <c r="D12">
         <v>4</v>
       </c>
       <c r="E12" t="s">
+        <v>39</v>
+      </c>
+      <c r="F12" t="s">
         <v>40</v>
       </c>
-      <c r="F12" t="s">
-        <v>41</v>
-      </c>
       <c r="G12" s="2" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="13" spans="1:7" ht="16.5" x14ac:dyDescent="0.3">
@@ -1107,19 +1107,19 @@
         <v>31</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>33</v>
+        <v>66</v>
       </c>
       <c r="D13">
         <v>5</v>
       </c>
       <c r="E13" t="s">
+        <v>41</v>
+      </c>
+      <c r="F13" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="F13" s="1" t="s">
-        <v>43</v>
-      </c>
       <c r="G13" s="2" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="14" spans="1:7" ht="16.5" x14ac:dyDescent="0.3">
@@ -1130,19 +1130,19 @@
         <v>31</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>33</v>
+        <v>66</v>
       </c>
       <c r="D14">
         <v>6</v>
       </c>
       <c r="E14" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="F14" t="s">
         <v>44</v>
       </c>
-      <c r="F14" t="s">
-        <v>45</v>
-      </c>
       <c r="G14" s="2" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="15" spans="1:7" ht="16.5" x14ac:dyDescent="0.3">
@@ -1153,16 +1153,16 @@
         <v>31</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>33</v>
+        <v>66</v>
       </c>
       <c r="D15">
         <v>7</v>
       </c>
       <c r="E15" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="F15" s="1" t="s">
         <v>46</v>
-      </c>
-      <c r="F15" s="1" t="s">
-        <v>47</v>
       </c>
       <c r="G15" s="2" t="s">
         <v>12</v>
@@ -1176,16 +1176,16 @@
         <v>31</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>33</v>
+        <v>66</v>
       </c>
       <c r="D16">
         <v>8</v>
       </c>
       <c r="E16" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="F16" s="1" t="s">
         <v>48</v>
-      </c>
-      <c r="F16" s="1" t="s">
-        <v>49</v>
       </c>
       <c r="G16" s="2" t="s">
         <v>12</v>
@@ -1199,16 +1199,16 @@
         <v>31</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>33</v>
+        <v>66</v>
       </c>
       <c r="D17">
         <v>9</v>
       </c>
       <c r="E17" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="F17" s="1" t="s">
         <v>50</v>
-      </c>
-      <c r="F17" s="1" t="s">
-        <v>51</v>
       </c>
       <c r="G17" s="2" t="s">
         <v>12</v>
@@ -1222,19 +1222,19 @@
         <v>31</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>33</v>
+        <v>66</v>
       </c>
       <c r="D18">
         <v>10</v>
       </c>
       <c r="E18" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="F18" t="s">
         <v>52</v>
       </c>
-      <c r="F18" t="s">
-        <v>53</v>
-      </c>
       <c r="G18" s="2" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
     </row>
     <row r="19" spans="1:7" ht="16.5" x14ac:dyDescent="0.3">
@@ -1245,19 +1245,19 @@
         <v>31</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>33</v>
+        <v>66</v>
       </c>
       <c r="D19">
         <v>11</v>
       </c>
       <c r="E19" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="F19" s="1" t="s">
         <v>54</v>
       </c>
-      <c r="F19" s="1" t="s">
-        <v>55</v>
-      </c>
       <c r="G19" s="2" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
     </row>
     <row r="20" spans="1:7" ht="16.5" x14ac:dyDescent="0.3">
@@ -1268,16 +1268,16 @@
         <v>31</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>33</v>
+        <v>66</v>
       </c>
       <c r="D20">
         <v>12</v>
       </c>
       <c r="E20" s="1" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="F20" s="1" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="G20" s="2" t="s">
         <v>22</v>
@@ -1291,19 +1291,19 @@
         <v>31</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>33</v>
+        <v>66</v>
       </c>
       <c r="D21">
         <v>13</v>
       </c>
       <c r="E21" s="1" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="F21" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="G21" s="2" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
     </row>
   </sheetData>

</xml_diff>